<commit_message>
Latest Code for Czechia
</commit_message>
<xml_diff>
--- a/Data/testData.xlsx
+++ b/Data/testData.xlsx
@@ -262,10 +262,10 @@
     <t>Slovakia</t>
   </si>
   <si>
-    <t>Cleve</t>
-  </si>
-  <si>
-    <t>Fay</t>
+    <t>Dandre</t>
+  </si>
+  <si>
+    <t>Bins-Hauck</t>
   </si>
   <si>
     <t>041/562 66 84</t>

</xml_diff>

<commit_message>
CZ completed, UK completed for staff 30
</commit_message>
<xml_diff>
--- a/Data/testData.xlsx
+++ b/Data/testData.xlsx
@@ -262,10 +262,10 @@
     <t>Slovakia</t>
   </si>
   <si>
-    <t>Dandre</t>
-  </si>
-  <si>
-    <t>Bins-Hauck</t>
+    <t>Blake</t>
+  </si>
+  <si>
+    <t>O'Keefe</t>
   </si>
   <si>
     <t>041/562 66 84</t>

</xml_diff>